<commit_message>
Updated notebooks with PyTorch CUDA support and improvements
</commit_message>
<xml_diff>
--- a/model_comparison_results.xlsx
+++ b/model_comparison_results.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>429.57</v>
+        <v>17.47</v>
       </c>
       <c r="C3" t="n">
         <v>0.986</v>
@@ -520,7 +520,7 @@
         <v>0.9935</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9953</v>
+        <v>0.9954</v>
       </c>
       <c r="H3" t="n">
         <v>111513</v>
@@ -533,10 +533,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62.01</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9827</v>
+        <v>0.9826</v>
       </c>
       <c r="D4" t="n">
         <v>0.9823</v>
@@ -561,13 +561,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>282.95</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9856</v>
+        <v>0.9855</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9844000000000001</v>
+        <v>0.9845</v>
       </c>
       <c r="E5" t="n">
         <v>0.9993</v>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>32.76</v>
+        <v>13.06</v>
       </c>
       <c r="C6" t="n">
         <v>0.983</v>
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>309.33</v>
+        <v>15.33</v>
       </c>
       <c r="C7" t="n">
         <v>0.9861</v>
@@ -645,19 +645,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>34.54</v>
+        <v>1.73</v>
       </c>
       <c r="C8" t="n">
         <v>0.9858</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9836</v>
+        <v>0.9835</v>
       </c>
       <c r="E8" t="n">
         <v>0.9984</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9933</v>
+        <v>0.9932</v>
       </c>
       <c r="G8" t="n">
         <v>0.9949</v>
@@ -673,13 +673,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>121.78</v>
+        <v>24.51</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9849</v>
+        <v>0.9848</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9843</v>
+        <v>0.9841</v>
       </c>
       <c r="E9" t="n">
         <v>0.9992</v>
@@ -688,7 +688,7 @@
         <v>0.9933999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9953</v>
+        <v>0.9952</v>
       </c>
       <c r="H9" t="n">
         <v>111513</v>
@@ -701,22 +701,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>20.41</v>
+        <v>2.41</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9627</v>
+        <v>0.9617</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9628</v>
+        <v>0.9618</v>
       </c>
       <c r="E10" t="n">
-        <v>0.986</v>
+        <v>0.9859</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9888</v>
+        <v>0.9886</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9874000000000001</v>
+        <v>0.9872</v>
       </c>
       <c r="H10" t="n">
         <v>111513</v>

</xml_diff>